<commit_message>
Fixed output filenames to match paper
</commit_message>
<xml_diff>
--- a/output/replication_package/05_static_did2s/models_did2s_static.xlsx
+++ b/output/replication_package/05_static_did2s/models_did2s_static.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\floods-and-mortgages\output\static_did2s\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\flood_events_residential_mortgage_performance\output\replication_package\05_static_did2s\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B6988A-37A9-4739-BD70-9B67618BDF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8E9C78-BA96-46BD-84D2-2E20619328D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18930" yWindow="2370" windowWidth="27870" windowHeight="13305" xr2:uid="{77D1EB07-154C-4469-B00F-902566111273}"/>
+    <workbookView xWindow="25830" yWindow="1890" windowWidth="24165" windowHeight="17655" xr2:uid="{77D1EB07-154C-4469-B00F-902566111273}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -365,42 +365,6 @@
     <t>HERMINE 90 delinq</t>
   </si>
   <si>
-    <t>Fig4-delinq90_harvey_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-delinq90_irma_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-delinq90_michael_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-delinq90_florence_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-delinq90_matthew_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-delinq90_hermine_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-foreclo_harvey_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-foreclo_irma_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-foreclo_michael_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-foreclo_florence_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-foreclo_matthew_static.png</t>
-  </si>
-  <si>
-    <t>Fig4-foreclo_hermine_static.png</t>
-  </si>
-  <si>
     <t>HARVEY foreclo</t>
   </si>
   <si>
@@ -453,6 +417,42 @@
   </si>
   <si>
     <t>~ 0 |  ID + date</t>
+  </si>
+  <si>
+    <t>FigS7-delinq90_michael_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-delinq90_florence_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-delinq90_matthew_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-delinq90_hermine_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-foreclo_harvey_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-foreclo_irma_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-foreclo_michael_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-foreclo_florence_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-foreclo_matthew_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-foreclo_hermine_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-delinq90_harvey_static.png</t>
+  </si>
+  <si>
+    <t>FigS7-delinq90_irma_static.png</t>
   </si>
 </sst>
 </file>
@@ -533,14 +533,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -856,7 +855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAE428A2-859C-4D47-8A62-EB930B793B17}">
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" bestFit="1" customWidth="1"/>
@@ -870,11 +869,10 @@
     <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="38.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="34.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="4"/>
+    <col min="12" max="12" width="34.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -908,7 +906,7 @@
       <c r="K1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>97</v>
       </c>
     </row>
@@ -946,7 +944,7 @@
       <c r="K2">
         <v>0</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -984,7 +982,7 @@
       <c r="K3">
         <v>1</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1022,7 +1020,7 @@
       <c r="K4">
         <v>2</v>
       </c>
-      <c r="L4" s="4" t="s">
+      <c r="L4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1060,7 +1058,7 @@
       <c r="K5">
         <v>3</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="L5" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1098,7 +1096,7 @@
       <c r="K6">
         <v>4</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1136,7 +1134,7 @@
       <c r="K7">
         <v>5</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="L7" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1174,7 +1172,7 @@
       <c r="K8">
         <v>0</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="L8" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1212,7 +1210,7 @@
       <c r="K9">
         <v>1</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="L9" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1250,7 +1248,7 @@
       <c r="K10">
         <v>2</v>
       </c>
-      <c r="L10" s="4" t="s">
+      <c r="L10" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1288,7 +1286,7 @@
       <c r="K11">
         <v>3</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="L11" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1326,7 +1324,7 @@
       <c r="K12">
         <v>4</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="L12" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1364,7 +1362,7 @@
       <c r="K13">
         <v>5</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="L13" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1402,7 +1400,7 @@
       <c r="K14">
         <v>0</v>
       </c>
-      <c r="L14" s="4" t="s">
+      <c r="L14" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1440,7 +1438,7 @@
       <c r="K15">
         <v>1</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="L15" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1478,7 +1476,7 @@
       <c r="K16">
         <v>2</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="L16" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1516,7 +1514,7 @@
       <c r="K17">
         <v>3</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="L17" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1554,7 +1552,7 @@
       <c r="K18">
         <v>4</v>
       </c>
-      <c r="L18" s="4" t="s">
+      <c r="L18" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1592,7 +1590,7 @@
       <c r="K19">
         <v>5</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="L19" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1600,34 +1598,34 @@
       <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="4" t="s">
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" t="s">
         <v>13</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J20" s="4" t="s">
+      <c r="H20" t="s">
+        <v>10</v>
+      </c>
+      <c r="I20" t="s">
+        <v>0</v>
+      </c>
+      <c r="J20" t="s">
         <v>95</v>
       </c>
-      <c r="L20" s="4" t="s">
+      <c r="L20" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1635,34 +1633,34 @@
       <c r="A21" s="2">
         <v>19</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" s="4" t="s">
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" t="s">
         <v>72</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" t="s">
         <v>70</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J21" s="4" t="s">
+      <c r="H21" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" t="s">
+        <v>0</v>
+      </c>
+      <c r="J21" t="s">
         <v>94</v>
       </c>
-      <c r="L21" s="4" t="s">
+      <c r="L21" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1700,7 +1698,7 @@
       <c r="K22">
         <v>6</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="L22" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1738,7 +1736,7 @@
       <c r="K23">
         <v>6</v>
       </c>
-      <c r="L23" s="4" t="s">
+      <c r="L23" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1771,9 +1769,9 @@
         <v>71</v>
       </c>
       <c r="J24" t="s">
-        <v>109</v>
-      </c>
-      <c r="L24" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="L24" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1806,9 +1804,9 @@
         <v>71</v>
       </c>
       <c r="J25" t="s">
-        <v>110</v>
-      </c>
-      <c r="L25" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="L25" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1841,9 +1839,9 @@
         <v>71</v>
       </c>
       <c r="J26" t="s">
-        <v>111</v>
-      </c>
-      <c r="L26" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="L26" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1876,9 +1874,9 @@
         <v>71</v>
       </c>
       <c r="J27" t="s">
-        <v>112</v>
-      </c>
-      <c r="L27" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L27" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1911,9 +1909,9 @@
         <v>71</v>
       </c>
       <c r="J28" t="s">
-        <v>113</v>
-      </c>
-      <c r="L28" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="L28" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1946,9 +1944,9 @@
         <v>71</v>
       </c>
       <c r="J29" t="s">
-        <v>114</v>
-      </c>
-      <c r="L29" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="L29" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1957,7 +1955,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C30" t="s">
         <v>51</v>
@@ -1981,9 +1979,9 @@
         <v>71</v>
       </c>
       <c r="J30" t="s">
-        <v>115</v>
-      </c>
-      <c r="L30" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="L30" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1992,7 +1990,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
         <v>51</v>
@@ -2016,9 +2014,9 @@
         <v>71</v>
       </c>
       <c r="J31" t="s">
-        <v>116</v>
-      </c>
-      <c r="L31" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L31" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2027,7 +2025,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C32" t="s">
         <v>51</v>
@@ -2051,9 +2049,9 @@
         <v>71</v>
       </c>
       <c r="J32" t="s">
-        <v>117</v>
-      </c>
-      <c r="L32" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="L32" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2062,7 +2060,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C33" t="s">
         <v>51</v>
@@ -2086,9 +2084,9 @@
         <v>71</v>
       </c>
       <c r="J33" t="s">
-        <v>118</v>
-      </c>
-      <c r="L33" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="L33" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2097,7 +2095,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C34" t="s">
         <v>51</v>
@@ -2121,9 +2119,9 @@
         <v>71</v>
       </c>
       <c r="J34" t="s">
-        <v>119</v>
-      </c>
-      <c r="L34" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="L34" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2132,7 +2130,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C35" t="s">
         <v>51</v>
@@ -2156,9 +2154,9 @@
         <v>71</v>
       </c>
       <c r="J35" t="s">
-        <v>120</v>
-      </c>
-      <c r="L35" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="L35" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2182,7 +2180,7 @@
         <v>13</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="H36" t="s">
         <v>10</v>
@@ -2196,7 +2194,7 @@
       <c r="K36">
         <v>7</v>
       </c>
-      <c r="L36" s="4" t="s">
+      <c r="L36" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2220,7 +2218,7 @@
         <v>13</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="H37" t="s">
         <v>10</v>
@@ -2234,7 +2232,7 @@
       <c r="K37">
         <v>7</v>
       </c>
-      <c r="L37" s="4" t="s">
+      <c r="L37" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2258,7 +2256,7 @@
         <v>13</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="H38" t="s">
         <v>10</v>
@@ -2272,7 +2270,7 @@
       <c r="K38">
         <v>7</v>
       </c>
-      <c r="L38" s="4" t="s">
+      <c r="L38" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2296,7 +2294,7 @@
         <v>13</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="H39" t="s">
         <v>10</v>
@@ -2310,7 +2308,7 @@
       <c r="K39">
         <v>7</v>
       </c>
-      <c r="L39" s="4" t="s">
+      <c r="L39" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2334,7 +2332,7 @@
         <v>13</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="H40" t="s">
         <v>10</v>
@@ -2348,7 +2346,7 @@
       <c r="K40">
         <v>7</v>
       </c>
-      <c r="L40" s="4" t="s">
+      <c r="L40" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2372,7 +2370,7 @@
         <v>13</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="H41" t="s">
         <v>10</v>
@@ -2386,7 +2384,7 @@
       <c r="K41">
         <v>7</v>
       </c>
-      <c r="L41" s="4" t="s">
+      <c r="L41" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2410,7 +2408,7 @@
         <v>13</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="H42" t="s">
         <v>10</v>
@@ -2424,7 +2422,7 @@
       <c r="K42">
         <v>7</v>
       </c>
-      <c r="L42" s="4" t="s">
+      <c r="L42" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2448,7 +2446,7 @@
         <v>13</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="H43" t="s">
         <v>10</v>
@@ -2462,7 +2460,7 @@
       <c r="K43">
         <v>7</v>
       </c>
-      <c r="L43" s="4" t="s">
+      <c r="L43" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2470,241 +2468,229 @@
       <c r="A44" s="2">
         <v>42</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D44" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="E44" s="7" t="s">
+      <c r="D44" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F44" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I44" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J44" s="7" t="s">
-        <v>131</v>
+      <c r="F44" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="K44">
         <v>0</v>
       </c>
-      <c r="L44" s="4" t="s">
-        <v>137</v>
+      <c r="L44" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>43</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E45" s="7" t="s">
+      <c r="D45" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F45" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J45" s="7" t="s">
-        <v>132</v>
+      <c r="F45" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>120</v>
       </c>
       <c r="K45">
         <v>1</v>
       </c>
-      <c r="L45" s="4" t="s">
-        <v>137</v>
+      <c r="L45" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>44</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="B46" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="C46" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D46" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E46" s="7" t="s">
+      <c r="D46" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F46" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I46" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J46" s="7" t="s">
-        <v>133</v>
+      <c r="F46" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>121</v>
       </c>
       <c r="K46">
         <v>2</v>
       </c>
-      <c r="L46" s="4" t="s">
-        <v>137</v>
+      <c r="L46" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B47" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="C47" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D47" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E47" s="7" t="s">
+      <c r="D47" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F47" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G47" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I47" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J47" s="7" t="s">
-        <v>134</v>
+      <c r="F47" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>122</v>
       </c>
       <c r="K47">
         <v>3</v>
       </c>
-      <c r="L47" s="4" t="s">
-        <v>137</v>
+      <c r="L47" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>46</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="B48" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C48" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D48" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E48" s="7" t="s">
+      <c r="D48" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F48" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I48" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J48" s="7" t="s">
-        <v>135</v>
+      <c r="F48" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="K48">
         <v>4</v>
       </c>
-      <c r="L48" s="4" t="s">
-        <v>137</v>
+      <c r="L48" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>47</v>
       </c>
-      <c r="B49" s="7" t="s">
+      <c r="B49" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C49" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D49" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E49" s="7" t="s">
+      <c r="D49" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E49" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F49" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I49" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J49" s="7" t="s">
-        <v>136</v>
+      <c r="F49" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>124</v>
       </c>
       <c r="K49">
         <v>5</v>
       </c>
-      <c r="L49" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="K50" s="4"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="K51" s="4"/>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="K52" s="4"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="K53" s="4"/>
+      <c r="L49" t="s">
+        <v>125</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>